<commit_message>
feat: close OCR clinical evidence gaps
</commit_message>
<xml_diff>
--- a/docs/schema/01_费用明细.xlsx
+++ b/docs/schema/01_费用明细.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -732,7 +732,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>单价</t>
+          <t>计价单位</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -742,29 +742,29 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>数字</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>单价 (元)</t>
+          <t>次/侧/眼/部位/小时等原始收费单位</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>790.00</t>
+          <t>次</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>pric / 单价（元）</t>
+          <t>unit / 单位 / 收费单位</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>规格</t>
+          <t>医嘱编号</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -779,24 +779,24 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>药品规格/耗材型号</t>
+          <t>费用行关联的医嘱 ID，可留空</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>5ml:0.1g</t>
+          <t>YZ-001</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>spec / 药品规格 / 耗材型号</t>
+          <t>order_id / YZID / 医嘱ID</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>项目编码</t>
+          <t>单价</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -806,29 +806,29 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数字</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>医保或院内项目编码</t>
+          <t>单价 (元)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>XJ01ABC123</t>
+          <t>790.00</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>medins_list_codg / med_list_codg / 医保编码 / 院内编码</t>
+          <t>pric / 单价（元）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>开单科室</t>
+          <t>规格</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -843,24 +843,24 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>申请/开单科室</t>
+          <t>药品规格/耗材型号</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>普外科</t>
+          <t>5ml:0.1g</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>acord_dept_name / 申请科室</t>
+          <t>spec / 药品规格 / 耗材型号</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>开单医生</t>
+          <t>项目编码</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -875,24 +875,24 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>申请/开单医生</t>
+          <t>医保或院内项目编码</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>张医生</t>
+          <t>XJ01ABC123</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>orders_dr_name / 申请医生</t>
+          <t>medins_list_codg / med_list_codg / 医保编码 / 院内编码</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>计费科室</t>
+          <t>开单科室</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -907,24 +907,24 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>执行/计费科室</t>
+          <t>申请/开单科室</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>药剂科</t>
+          <t>普外科</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>bilg_dept_name / 执行科室</t>
+          <t>acord_dept_name / 申请科室</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>计费医生</t>
+          <t>开单医生</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -939,47 +939,111 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>执行/计费医生</t>
+          <t>申请/开单医生</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>李医生</t>
+          <t>张医生</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>bilg_dr_name / 执行医生</t>
+          <t>orders_dr_name / 申请医生</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>计费科室</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>执行/计费科室</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>药剂科</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>bilg_dept_name / 执行科室</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>计费医生</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>执行/计费医生</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>李医生</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>bilg_dr_name / 执行医生</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>药品通用名</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>可选</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>文本</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>药品通用名 (区别于收费项目名/商品名)</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>利多卡因</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>prodname / 通用名 / 商品名</t>
         </is>
@@ -1001,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1018,6 +1082,8 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1053,40 +1119,50 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
+          <t>计价单位</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>医嘱编号</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>单价</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>规格</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>项目编码</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>开单科室</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>开单医生</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>计费科室</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>计费医生</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>药品通用名</t>
         </is>

</xml_diff>